<commit_message>
Miscellaneous minor fixes and improvements:
- Added pandas ad dependency to pyproject.toml
- stats module: made mean load factor explicit by adding a parameter to
  the standard markov matrix sampler function
- stats module: made fatigue class distribution parameters explicit in
  the standard bolt fatigue curve sampler function
- validation: adapdet the L-Flange gen-cases.py script to the latest
  breaking changes
</commit_message>
<xml_diff>
--- a/validations/flangesegments.PolynomialLFlangeSegment/Case_1_D7500_L_Tilt-0p00deg_ShapeFactor-1p00_Fv2800kN_ShellStiff-Interp.xlsx
+++ b/validations/flangesegments.PolynomialLFlangeSegment/Case_1_D7500_L_Tilt-0p00deg_ShapeFactor-1p00_Fv2800kN_ShellStiff-Interp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarcelloB\mdb\!Progetti\!KCI\!SP2200052 - Bolt &amp; Beautiful\!pyflange-package\validations\flangesegments.PolynomialLFlangeSegment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MSYS2\home\marcello\mdb\!Progetti\!KCI\Tools\pyflange\validations\flangesegments.PolynomialLFlangeSegment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86975629-807C-4B02-9820-943D2B15CB45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099A34E8-F154-428B-ABB8-A7F3787DD7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-7200" windowWidth="29040" windowHeight="18240" activeTab="1" xr2:uid="{710C990D-69B5-462C-923E-A1886280CCCB}"/>
+    <workbookView xWindow="28680" yWindow="-8250" windowWidth="29040" windowHeight="18240" activeTab="1" xr2:uid="{710C990D-69B5-462C-923E-A1886280CCCB}"/>
   </bookViews>
   <sheets>
     <sheet name="Comparison" sheetId="16" r:id="rId1"/>
@@ -5892,6 +5892,15 @@
     <xf numFmtId="165" fontId="11" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5919,17 +5928,8 @@
     <xf numFmtId="0" fontId="26" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="13" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -7001,7 +7001,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -7056,6 +7056,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7063,7 +7064,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7959,7 +7959,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -8014,6 +8014,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8021,7 +8022,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8916,7 +8916,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -8971,6 +8971,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8978,7 +8979,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9874,7 +9874,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -9929,6 +9929,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9936,7 +9937,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10831,7 +10831,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -10886,6 +10886,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10893,7 +10894,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11789,7 +11789,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -11844,6 +11844,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11851,7 +11852,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12746,7 +12746,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -12801,6 +12801,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12808,7 +12809,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13704,7 +13704,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13759,6 +13759,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13766,7 +13767,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14327,6 +14327,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14334,7 +14335,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -20093,7 +20093,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-NL" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-GB" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -20250,7 +20250,7 @@
                 <a:defRPr sz="1000"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-NL" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-GB" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
                   </a:solidFill>
@@ -23172,32 +23172,32 @@
       <c r="K2" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="54.75" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A3" s="180" t="s">
+      <c r="A3" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="181"/>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
-      <c r="H3" s="181"/>
-      <c r="I3" s="181"/>
-      <c r="J3" s="181"/>
-      <c r="K3" s="181"/>
+      <c r="B3" s="184"/>
+      <c r="C3" s="184"/>
+      <c r="D3" s="184"/>
+      <c r="E3" s="184"/>
+      <c r="F3" s="184"/>
+      <c r="G3" s="184"/>
+      <c r="H3" s="184"/>
+      <c r="I3" s="184"/>
+      <c r="J3" s="184"/>
+      <c r="K3" s="184"/>
     </row>
     <row r="4" spans="1:15" s="46" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="182" t="s">
+      <c r="B4" s="185" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="182"/>
-      <c r="D4" s="182"/>
-      <c r="E4" s="182"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
+      <c r="F4" s="185"/>
+      <c r="G4" s="185"/>
       <c r="H4" s="47" t="s">
         <v>14</v>
       </c>
@@ -23213,12 +23213,12 @@
     </row>
     <row r="5" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A5" s="45"/>
-      <c r="B5" s="183"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
-      <c r="E5" s="184"/>
-      <c r="F5" s="184"/>
-      <c r="G5" s="185"/>
+      <c r="B5" s="186"/>
+      <c r="C5" s="187"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="187"/>
+      <c r="F5" s="187"/>
+      <c r="G5" s="188"/>
       <c r="H5" s="44"/>
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
@@ -23226,12 +23226,12 @@
     </row>
     <row r="6" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A6" s="45"/>
-      <c r="B6" s="183"/>
-      <c r="C6" s="184"/>
-      <c r="D6" s="184"/>
-      <c r="E6" s="184"/>
-      <c r="F6" s="184"/>
-      <c r="G6" s="185"/>
+      <c r="B6" s="186"/>
+      <c r="C6" s="187"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="187"/>
+      <c r="G6" s="188"/>
       <c r="H6" s="44"/>
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
@@ -23239,12 +23239,12 @@
     </row>
     <row r="7" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A7" s="45"/>
-      <c r="B7" s="183"/>
-      <c r="C7" s="184"/>
-      <c r="D7" s="184"/>
-      <c r="E7" s="184"/>
-      <c r="F7" s="184"/>
-      <c r="G7" s="185"/>
+      <c r="B7" s="186"/>
+      <c r="C7" s="187"/>
+      <c r="D7" s="187"/>
+      <c r="E7" s="187"/>
+      <c r="F7" s="187"/>
+      <c r="G7" s="188"/>
       <c r="H7" s="44"/>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
@@ -23252,12 +23252,12 @@
     </row>
     <row r="8" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A8" s="45"/>
-      <c r="B8" s="183"/>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
-      <c r="F8" s="184"/>
-      <c r="G8" s="185"/>
+      <c r="B8" s="186"/>
+      <c r="C8" s="187"/>
+      <c r="D8" s="187"/>
+      <c r="E8" s="187"/>
+      <c r="F8" s="187"/>
+      <c r="G8" s="188"/>
       <c r="H8" s="44"/>
       <c r="I8" s="43"/>
       <c r="J8" s="43"/>
@@ -23265,12 +23265,12 @@
     </row>
     <row r="9" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A9" s="45"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="184"/>
-      <c r="D9" s="184"/>
-      <c r="E9" s="184"/>
-      <c r="F9" s="184"/>
-      <c r="G9" s="185"/>
+      <c r="B9" s="186"/>
+      <c r="C9" s="187"/>
+      <c r="D9" s="187"/>
+      <c r="E9" s="187"/>
+      <c r="F9" s="187"/>
+      <c r="G9" s="188"/>
       <c r="H9" s="44"/>
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
@@ -23318,112 +23318,112 @@
     </row>
     <row r="13" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A13" s="87"/>
-      <c r="B13" s="186" t="s">
+      <c r="B13" s="179" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="186"/>
-      <c r="D13" s="188" t="s">
+      <c r="C13" s="179"/>
+      <c r="D13" s="178" t="s">
         <v>101</v>
       </c>
-      <c r="E13" s="188"/>
-      <c r="F13" s="188"/>
-      <c r="G13" s="188"/>
-      <c r="H13" s="188"/>
-      <c r="I13" s="188"/>
-      <c r="J13" s="188"/>
-      <c r="K13" s="188"/>
+      <c r="E13" s="178"/>
+      <c r="F13" s="178"/>
+      <c r="G13" s="178"/>
+      <c r="H13" s="178"/>
+      <c r="I13" s="178"/>
+      <c r="J13" s="178"/>
+      <c r="K13" s="178"/>
       <c r="L13" s="86"/>
     </row>
     <row r="14" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A14" s="87"/>
-      <c r="B14" s="186" t="s">
+      <c r="B14" s="179" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="186"/>
-      <c r="D14" s="188" t="s">
+      <c r="C14" s="179"/>
+      <c r="D14" s="178" t="s">
         <v>103</v>
       </c>
-      <c r="E14" s="188"/>
-      <c r="F14" s="188"/>
-      <c r="G14" s="188"/>
-      <c r="H14" s="188"/>
-      <c r="I14" s="188"/>
-      <c r="J14" s="188"/>
-      <c r="K14" s="188"/>
+      <c r="E14" s="178"/>
+      <c r="F14" s="178"/>
+      <c r="G14" s="178"/>
+      <c r="H14" s="178"/>
+      <c r="I14" s="178"/>
+      <c r="J14" s="178"/>
+      <c r="K14" s="178"/>
       <c r="L14" s="86"/>
     </row>
     <row r="15" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A15" s="87"/>
-      <c r="B15" s="186" t="s">
+      <c r="B15" s="179" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="186"/>
-      <c r="D15" s="188" t="s">
+      <c r="C15" s="179"/>
+      <c r="D15" s="178" t="s">
         <v>102</v>
       </c>
-      <c r="E15" s="188"/>
-      <c r="F15" s="188"/>
-      <c r="G15" s="188"/>
-      <c r="H15" s="188"/>
-      <c r="I15" s="188"/>
-      <c r="J15" s="188"/>
-      <c r="K15" s="188"/>
+      <c r="E15" s="178"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="178"/>
+      <c r="H15" s="178"/>
+      <c r="I15" s="178"/>
+      <c r="J15" s="178"/>
+      <c r="K15" s="178"/>
       <c r="L15" s="86"/>
     </row>
     <row r="16" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A16" s="87"/>
-      <c r="B16" s="186" t="s">
+      <c r="B16" s="179" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="186"/>
-      <c r="D16" s="188" t="str">
+      <c r="C16" s="179"/>
+      <c r="D16" s="178" t="str">
         <f>Title</f>
         <v>Flange Segment Analytical Model for 30° gap size</v>
       </c>
-      <c r="E16" s="188"/>
-      <c r="F16" s="188"/>
-      <c r="G16" s="188"/>
-      <c r="H16" s="188"/>
-      <c r="I16" s="188"/>
-      <c r="J16" s="188"/>
-      <c r="K16" s="188"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="178"/>
+      <c r="G16" s="178"/>
+      <c r="H16" s="178"/>
+      <c r="I16" s="178"/>
+      <c r="J16" s="178"/>
+      <c r="K16" s="178"/>
       <c r="L16" s="86"/>
       <c r="M16" s="88"/>
     </row>
     <row r="17" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A17" s="87"/>
-      <c r="B17" s="186" t="s">
+      <c r="B17" s="179" t="s">
         <v>96</v>
       </c>
-      <c r="C17" s="186"/>
-      <c r="D17" s="189" t="s">
+      <c r="C17" s="179"/>
+      <c r="D17" s="177" t="s">
         <v>324</v>
       </c>
-      <c r="E17" s="188"/>
-      <c r="F17" s="188"/>
-      <c r="G17" s="188"/>
-      <c r="H17" s="188"/>
-      <c r="I17" s="188"/>
-      <c r="J17" s="188"/>
-      <c r="K17" s="188"/>
+      <c r="E17" s="178"/>
+      <c r="F17" s="178"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="178"/>
+      <c r="I17" s="178"/>
+      <c r="J17" s="178"/>
+      <c r="K17" s="178"/>
       <c r="L17" s="86"/>
     </row>
     <row r="18" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A18" s="87"/>
-      <c r="B18" s="186" t="s">
+      <c r="B18" s="179" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="186"/>
-      <c r="D18" s="187">
+      <c r="C18" s="179"/>
+      <c r="D18" s="189">
         <v>45432</v>
       </c>
-      <c r="E18" s="187"/>
-      <c r="F18" s="187"/>
-      <c r="G18" s="187"/>
-      <c r="H18" s="187"/>
-      <c r="I18" s="187"/>
-      <c r="J18" s="187"/>
-      <c r="K18" s="187"/>
+      <c r="E18" s="189"/>
+      <c r="F18" s="189"/>
+      <c r="G18" s="189"/>
+      <c r="H18" s="189"/>
+      <c r="I18" s="189"/>
+      <c r="J18" s="189"/>
+      <c r="K18" s="189"/>
       <c r="L18" s="86"/>
     </row>
     <row r="19" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
@@ -23611,16 +23611,16 @@
     </row>
     <row r="28" spans="1:22" s="18" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A28" s="21"/>
-      <c r="B28" s="177"/>
-      <c r="C28" s="178"/>
-      <c r="D28" s="178"/>
-      <c r="E28" s="178"/>
-      <c r="F28" s="178"/>
-      <c r="G28" s="178"/>
-      <c r="H28" s="178"/>
-      <c r="I28" s="178"/>
-      <c r="J28" s="178"/>
-      <c r="K28" s="179"/>
+      <c r="B28" s="180"/>
+      <c r="C28" s="181"/>
+      <c r="D28" s="181"/>
+      <c r="E28" s="181"/>
+      <c r="F28" s="181"/>
+      <c r="G28" s="181"/>
+      <c r="H28" s="181"/>
+      <c r="I28" s="181"/>
+      <c r="J28" s="181"/>
+      <c r="K28" s="182"/>
       <c r="L28" s="20"/>
       <c r="M28" s="19"/>
       <c r="N28" s="19"/>
@@ -27616,16 +27616,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:K15"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B28:K28"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B18:C18"/>
@@ -27636,6 +27626,16 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:K16"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:K15"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B28:K28"/>
   </mergeCells>
   <conditionalFormatting sqref="K64">
     <cfRule type="cellIs" dxfId="11" priority="5" stopIfTrue="1" operator="between">
@@ -27716,32 +27716,32 @@
       <c r="K2" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="54.75" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A3" s="180" t="s">
+      <c r="A3" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="181"/>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
-      <c r="H3" s="181"/>
-      <c r="I3" s="181"/>
-      <c r="J3" s="181"/>
-      <c r="K3" s="181"/>
+      <c r="B3" s="184"/>
+      <c r="C3" s="184"/>
+      <c r="D3" s="184"/>
+      <c r="E3" s="184"/>
+      <c r="F3" s="184"/>
+      <c r="G3" s="184"/>
+      <c r="H3" s="184"/>
+      <c r="I3" s="184"/>
+      <c r="J3" s="184"/>
+      <c r="K3" s="184"/>
     </row>
     <row r="4" spans="1:15" s="46" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="182" t="s">
+      <c r="B4" s="185" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="182"/>
-      <c r="D4" s="182"/>
-      <c r="E4" s="182"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
+      <c r="F4" s="185"/>
+      <c r="G4" s="185"/>
       <c r="H4" s="47" t="s">
         <v>14</v>
       </c>
@@ -27757,12 +27757,12 @@
     </row>
     <row r="5" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A5" s="45"/>
-      <c r="B5" s="183"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
-      <c r="E5" s="184"/>
-      <c r="F5" s="184"/>
-      <c r="G5" s="185"/>
+      <c r="B5" s="186"/>
+      <c r="C5" s="187"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="187"/>
+      <c r="F5" s="187"/>
+      <c r="G5" s="188"/>
       <c r="H5" s="44"/>
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
@@ -27770,12 +27770,12 @@
     </row>
     <row r="6" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A6" s="45"/>
-      <c r="B6" s="183"/>
-      <c r="C6" s="184"/>
-      <c r="D6" s="184"/>
-      <c r="E6" s="184"/>
-      <c r="F6" s="184"/>
-      <c r="G6" s="185"/>
+      <c r="B6" s="186"/>
+      <c r="C6" s="187"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="187"/>
+      <c r="G6" s="188"/>
       <c r="H6" s="44"/>
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
@@ -27783,12 +27783,12 @@
     </row>
     <row r="7" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A7" s="45"/>
-      <c r="B7" s="183"/>
-      <c r="C7" s="184"/>
-      <c r="D7" s="184"/>
-      <c r="E7" s="184"/>
-      <c r="F7" s="184"/>
-      <c r="G7" s="185"/>
+      <c r="B7" s="186"/>
+      <c r="C7" s="187"/>
+      <c r="D7" s="187"/>
+      <c r="E7" s="187"/>
+      <c r="F7" s="187"/>
+      <c r="G7" s="188"/>
       <c r="H7" s="44"/>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
@@ -27796,12 +27796,12 @@
     </row>
     <row r="8" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A8" s="45"/>
-      <c r="B8" s="183"/>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
-      <c r="F8" s="184"/>
-      <c r="G8" s="185"/>
+      <c r="B8" s="186"/>
+      <c r="C8" s="187"/>
+      <c r="D8" s="187"/>
+      <c r="E8" s="187"/>
+      <c r="F8" s="187"/>
+      <c r="G8" s="188"/>
       <c r="H8" s="44"/>
       <c r="I8" s="43"/>
       <c r="J8" s="43"/>
@@ -27809,12 +27809,12 @@
     </row>
     <row r="9" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A9" s="45"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="184"/>
-      <c r="D9" s="184"/>
-      <c r="E9" s="184"/>
-      <c r="F9" s="184"/>
-      <c r="G9" s="185"/>
+      <c r="B9" s="186"/>
+      <c r="C9" s="187"/>
+      <c r="D9" s="187"/>
+      <c r="E9" s="187"/>
+      <c r="F9" s="187"/>
+      <c r="G9" s="188"/>
       <c r="H9" s="44"/>
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
@@ -27862,117 +27862,117 @@
     </row>
     <row r="13" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A13" s="87"/>
-      <c r="B13" s="186" t="s">
+      <c r="B13" s="179" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="186"/>
-      <c r="D13" s="188" t="str">
+      <c r="C13" s="179"/>
+      <c r="D13" s="178" t="str">
         <f>PyFlange_Gap30deg!D13</f>
         <v>SP2200052</v>
       </c>
-      <c r="E13" s="188"/>
-      <c r="F13" s="188"/>
-      <c r="G13" s="188"/>
-      <c r="H13" s="188"/>
-      <c r="I13" s="188"/>
-      <c r="J13" s="188"/>
-      <c r="K13" s="188"/>
+      <c r="E13" s="178"/>
+      <c r="F13" s="178"/>
+      <c r="G13" s="178"/>
+      <c r="H13" s="178"/>
+      <c r="I13" s="178"/>
+      <c r="J13" s="178"/>
+      <c r="K13" s="178"/>
       <c r="L13" s="86"/>
     </row>
     <row r="14" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A14" s="87"/>
-      <c r="B14" s="186" t="s">
+      <c r="B14" s="179" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="186"/>
-      <c r="D14" s="188" t="str">
+      <c r="C14" s="179"/>
+      <c r="D14" s="178" t="str">
         <f>PyFlange_Gap30deg!D14</f>
         <v>Stichting GROW</v>
       </c>
-      <c r="E14" s="188"/>
-      <c r="F14" s="188"/>
-      <c r="G14" s="188"/>
-      <c r="H14" s="188"/>
-      <c r="I14" s="188"/>
-      <c r="J14" s="188"/>
-      <c r="K14" s="188"/>
+      <c r="E14" s="178"/>
+      <c r="F14" s="178"/>
+      <c r="G14" s="178"/>
+      <c r="H14" s="178"/>
+      <c r="I14" s="178"/>
+      <c r="J14" s="178"/>
+      <c r="K14" s="178"/>
       <c r="L14" s="86"/>
     </row>
     <row r="15" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A15" s="87"/>
-      <c r="B15" s="186" t="s">
+      <c r="B15" s="179" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="186"/>
-      <c r="D15" s="188" t="str">
+      <c r="C15" s="179"/>
+      <c r="D15" s="178" t="str">
         <f>PyFlange_Gap30deg!D15</f>
         <v>Bolt and Beautiful</v>
       </c>
-      <c r="E15" s="188"/>
-      <c r="F15" s="188"/>
-      <c r="G15" s="188"/>
-      <c r="H15" s="188"/>
-      <c r="I15" s="188"/>
-      <c r="J15" s="188"/>
-      <c r="K15" s="188"/>
+      <c r="E15" s="178"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="178"/>
+      <c r="H15" s="178"/>
+      <c r="I15" s="178"/>
+      <c r="J15" s="178"/>
+      <c r="K15" s="178"/>
       <c r="L15" s="86"/>
     </row>
     <row r="16" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A16" s="87"/>
-      <c r="B16" s="186" t="s">
+      <c r="B16" s="179" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="186"/>
-      <c r="D16" s="188" t="str">
+      <c r="C16" s="179"/>
+      <c r="D16" s="178" t="str">
         <f>Title</f>
         <v>Flange Segment Analytical Model for 60° gap size</v>
       </c>
-      <c r="E16" s="188"/>
-      <c r="F16" s="188"/>
-      <c r="G16" s="188"/>
-      <c r="H16" s="188"/>
-      <c r="I16" s="188"/>
-      <c r="J16" s="188"/>
-      <c r="K16" s="188"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="178"/>
+      <c r="G16" s="178"/>
+      <c r="H16" s="178"/>
+      <c r="I16" s="178"/>
+      <c r="J16" s="178"/>
+      <c r="K16" s="178"/>
       <c r="L16" s="86"/>
       <c r="M16" s="88"/>
     </row>
     <row r="17" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A17" s="87"/>
-      <c r="B17" s="186" t="s">
+      <c r="B17" s="179" t="s">
         <v>96</v>
       </c>
-      <c r="C17" s="186"/>
-      <c r="D17" s="188" t="str">
+      <c r="C17" s="179"/>
+      <c r="D17" s="178" t="str">
         <f>PyFlange_Gap30deg!D17</f>
         <v>0.10</v>
       </c>
-      <c r="E17" s="188"/>
-      <c r="F17" s="188"/>
-      <c r="G17" s="188"/>
-      <c r="H17" s="188"/>
-      <c r="I17" s="188"/>
-      <c r="J17" s="188"/>
-      <c r="K17" s="188"/>
+      <c r="E17" s="178"/>
+      <c r="F17" s="178"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="178"/>
+      <c r="I17" s="178"/>
+      <c r="J17" s="178"/>
+      <c r="K17" s="178"/>
       <c r="L17" s="86"/>
     </row>
     <row r="18" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A18" s="87"/>
-      <c r="B18" s="186" t="s">
+      <c r="B18" s="179" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="186"/>
-      <c r="D18" s="187">
+      <c r="C18" s="179"/>
+      <c r="D18" s="189">
         <f>PyFlange_Gap30deg!D18</f>
         <v>45432</v>
       </c>
-      <c r="E18" s="187"/>
-      <c r="F18" s="187"/>
-      <c r="G18" s="187"/>
-      <c r="H18" s="187"/>
-      <c r="I18" s="187"/>
-      <c r="J18" s="187"/>
-      <c r="K18" s="187"/>
+      <c r="E18" s="189"/>
+      <c r="F18" s="189"/>
+      <c r="G18" s="189"/>
+      <c r="H18" s="189"/>
+      <c r="I18" s="189"/>
+      <c r="J18" s="189"/>
+      <c r="K18" s="189"/>
       <c r="L18" s="86"/>
     </row>
     <row r="19" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
@@ -28160,16 +28160,16 @@
     </row>
     <row r="28" spans="1:22" s="18" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A28" s="21"/>
-      <c r="B28" s="177"/>
-      <c r="C28" s="178"/>
-      <c r="D28" s="178"/>
-      <c r="E28" s="178"/>
-      <c r="F28" s="178"/>
-      <c r="G28" s="178"/>
-      <c r="H28" s="178"/>
-      <c r="I28" s="178"/>
-      <c r="J28" s="178"/>
-      <c r="K28" s="179"/>
+      <c r="B28" s="180"/>
+      <c r="C28" s="181"/>
+      <c r="D28" s="181"/>
+      <c r="E28" s="181"/>
+      <c r="F28" s="181"/>
+      <c r="G28" s="181"/>
+      <c r="H28" s="181"/>
+      <c r="I28" s="181"/>
+      <c r="J28" s="181"/>
+      <c r="K28" s="182"/>
       <c r="L28" s="20"/>
       <c r="M28" s="19"/>
       <c r="N28" s="19"/>
@@ -32138,6 +32138,13 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B28:K28"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:K16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:K18"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="D15:K15"/>
     <mergeCell ref="A3:K3"/>
@@ -32151,13 +32158,6 @@
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="D14:K14"/>
-    <mergeCell ref="B28:K28"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:K16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:K18"/>
   </mergeCells>
   <conditionalFormatting sqref="K64">
     <cfRule type="cellIs" dxfId="8" priority="3" stopIfTrue="1" operator="between">
@@ -32238,32 +32238,32 @@
       <c r="K2" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="54.75" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A3" s="180" t="s">
+      <c r="A3" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="181"/>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
-      <c r="H3" s="181"/>
-      <c r="I3" s="181"/>
-      <c r="J3" s="181"/>
-      <c r="K3" s="181"/>
+      <c r="B3" s="184"/>
+      <c r="C3" s="184"/>
+      <c r="D3" s="184"/>
+      <c r="E3" s="184"/>
+      <c r="F3" s="184"/>
+      <c r="G3" s="184"/>
+      <c r="H3" s="184"/>
+      <c r="I3" s="184"/>
+      <c r="J3" s="184"/>
+      <c r="K3" s="184"/>
     </row>
     <row r="4" spans="1:15" s="46" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="182" t="s">
+      <c r="B4" s="185" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="182"/>
-      <c r="D4" s="182"/>
-      <c r="E4" s="182"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
+      <c r="F4" s="185"/>
+      <c r="G4" s="185"/>
       <c r="H4" s="47" t="s">
         <v>14</v>
       </c>
@@ -32279,12 +32279,12 @@
     </row>
     <row r="5" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A5" s="45"/>
-      <c r="B5" s="183"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
-      <c r="E5" s="184"/>
-      <c r="F5" s="184"/>
-      <c r="G5" s="185"/>
+      <c r="B5" s="186"/>
+      <c r="C5" s="187"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="187"/>
+      <c r="F5" s="187"/>
+      <c r="G5" s="188"/>
       <c r="H5" s="44"/>
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
@@ -32292,12 +32292,12 @@
     </row>
     <row r="6" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A6" s="45"/>
-      <c r="B6" s="183"/>
-      <c r="C6" s="184"/>
-      <c r="D6" s="184"/>
-      <c r="E6" s="184"/>
-      <c r="F6" s="184"/>
-      <c r="G6" s="185"/>
+      <c r="B6" s="186"/>
+      <c r="C6" s="187"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="187"/>
+      <c r="G6" s="188"/>
       <c r="H6" s="44"/>
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
@@ -32305,12 +32305,12 @@
     </row>
     <row r="7" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A7" s="45"/>
-      <c r="B7" s="183"/>
-      <c r="C7" s="184"/>
-      <c r="D7" s="184"/>
-      <c r="E7" s="184"/>
-      <c r="F7" s="184"/>
-      <c r="G7" s="185"/>
+      <c r="B7" s="186"/>
+      <c r="C7" s="187"/>
+      <c r="D7" s="187"/>
+      <c r="E7" s="187"/>
+      <c r="F7" s="187"/>
+      <c r="G7" s="188"/>
       <c r="H7" s="44"/>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
@@ -32318,12 +32318,12 @@
     </row>
     <row r="8" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A8" s="45"/>
-      <c r="B8" s="183"/>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
-      <c r="F8" s="184"/>
-      <c r="G8" s="185"/>
+      <c r="B8" s="186"/>
+      <c r="C8" s="187"/>
+      <c r="D8" s="187"/>
+      <c r="E8" s="187"/>
+      <c r="F8" s="187"/>
+      <c r="G8" s="188"/>
       <c r="H8" s="44"/>
       <c r="I8" s="43"/>
       <c r="J8" s="43"/>
@@ -32331,12 +32331,12 @@
     </row>
     <row r="9" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A9" s="45"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="184"/>
-      <c r="D9" s="184"/>
-      <c r="E9" s="184"/>
-      <c r="F9" s="184"/>
-      <c r="G9" s="185"/>
+      <c r="B9" s="186"/>
+      <c r="C9" s="187"/>
+      <c r="D9" s="187"/>
+      <c r="E9" s="187"/>
+      <c r="F9" s="187"/>
+      <c r="G9" s="188"/>
       <c r="H9" s="44"/>
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
@@ -32384,117 +32384,117 @@
     </row>
     <row r="13" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A13" s="87"/>
-      <c r="B13" s="186" t="s">
+      <c r="B13" s="179" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="186"/>
-      <c r="D13" s="188" t="str">
+      <c r="C13" s="179"/>
+      <c r="D13" s="178" t="str">
         <f>PyFlange_Gap30deg!D13</f>
         <v>SP2200052</v>
       </c>
-      <c r="E13" s="188"/>
-      <c r="F13" s="188"/>
-      <c r="G13" s="188"/>
-      <c r="H13" s="188"/>
-      <c r="I13" s="188"/>
-      <c r="J13" s="188"/>
-      <c r="K13" s="188"/>
+      <c r="E13" s="178"/>
+      <c r="F13" s="178"/>
+      <c r="G13" s="178"/>
+      <c r="H13" s="178"/>
+      <c r="I13" s="178"/>
+      <c r="J13" s="178"/>
+      <c r="K13" s="178"/>
       <c r="L13" s="86"/>
     </row>
     <row r="14" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A14" s="87"/>
-      <c r="B14" s="186" t="s">
+      <c r="B14" s="179" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="186"/>
-      <c r="D14" s="188" t="str">
+      <c r="C14" s="179"/>
+      <c r="D14" s="178" t="str">
         <f>PyFlange_Gap30deg!D14</f>
         <v>Stichting GROW</v>
       </c>
-      <c r="E14" s="188"/>
-      <c r="F14" s="188"/>
-      <c r="G14" s="188"/>
-      <c r="H14" s="188"/>
-      <c r="I14" s="188"/>
-      <c r="J14" s="188"/>
-      <c r="K14" s="188"/>
+      <c r="E14" s="178"/>
+      <c r="F14" s="178"/>
+      <c r="G14" s="178"/>
+      <c r="H14" s="178"/>
+      <c r="I14" s="178"/>
+      <c r="J14" s="178"/>
+      <c r="K14" s="178"/>
       <c r="L14" s="86"/>
     </row>
     <row r="15" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A15" s="87"/>
-      <c r="B15" s="186" t="s">
+      <c r="B15" s="179" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="186"/>
-      <c r="D15" s="188" t="str">
+      <c r="C15" s="179"/>
+      <c r="D15" s="178" t="str">
         <f>PyFlange_Gap30deg!D15</f>
         <v>Bolt and Beautiful</v>
       </c>
-      <c r="E15" s="188"/>
-      <c r="F15" s="188"/>
-      <c r="G15" s="188"/>
-      <c r="H15" s="188"/>
-      <c r="I15" s="188"/>
-      <c r="J15" s="188"/>
-      <c r="K15" s="188"/>
+      <c r="E15" s="178"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="178"/>
+      <c r="H15" s="178"/>
+      <c r="I15" s="178"/>
+      <c r="J15" s="178"/>
+      <c r="K15" s="178"/>
       <c r="L15" s="86"/>
     </row>
     <row r="16" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A16" s="87"/>
-      <c r="B16" s="186" t="s">
+      <c r="B16" s="179" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="186"/>
-      <c r="D16" s="188" t="str">
+      <c r="C16" s="179"/>
+      <c r="D16" s="178" t="str">
         <f>Title</f>
         <v>Flange Segment Analytical Model for 90° gap size</v>
       </c>
-      <c r="E16" s="188"/>
-      <c r="F16" s="188"/>
-      <c r="G16" s="188"/>
-      <c r="H16" s="188"/>
-      <c r="I16" s="188"/>
-      <c r="J16" s="188"/>
-      <c r="K16" s="188"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="178"/>
+      <c r="G16" s="178"/>
+      <c r="H16" s="178"/>
+      <c r="I16" s="178"/>
+      <c r="J16" s="178"/>
+      <c r="K16" s="178"/>
       <c r="L16" s="86"/>
       <c r="M16" s="88"/>
     </row>
     <row r="17" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A17" s="87"/>
-      <c r="B17" s="186" t="s">
+      <c r="B17" s="179" t="s">
         <v>96</v>
       </c>
-      <c r="C17" s="186"/>
-      <c r="D17" s="188" t="str">
+      <c r="C17" s="179"/>
+      <c r="D17" s="178" t="str">
         <f>PyFlange_Gap30deg!D17</f>
         <v>0.10</v>
       </c>
-      <c r="E17" s="188"/>
-      <c r="F17" s="188"/>
-      <c r="G17" s="188"/>
-      <c r="H17" s="188"/>
-      <c r="I17" s="188"/>
-      <c r="J17" s="188"/>
-      <c r="K17" s="188"/>
+      <c r="E17" s="178"/>
+      <c r="F17" s="178"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="178"/>
+      <c r="I17" s="178"/>
+      <c r="J17" s="178"/>
+      <c r="K17" s="178"/>
       <c r="L17" s="86"/>
     </row>
     <row r="18" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A18" s="87"/>
-      <c r="B18" s="186" t="s">
+      <c r="B18" s="179" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="186"/>
-      <c r="D18" s="187">
+      <c r="C18" s="179"/>
+      <c r="D18" s="189">
         <f>PyFlange_Gap30deg!D18</f>
         <v>45432</v>
       </c>
-      <c r="E18" s="187"/>
-      <c r="F18" s="187"/>
-      <c r="G18" s="187"/>
-      <c r="H18" s="187"/>
-      <c r="I18" s="187"/>
-      <c r="J18" s="187"/>
-      <c r="K18" s="187"/>
+      <c r="E18" s="189"/>
+      <c r="F18" s="189"/>
+      <c r="G18" s="189"/>
+      <c r="H18" s="189"/>
+      <c r="I18" s="189"/>
+      <c r="J18" s="189"/>
+      <c r="K18" s="189"/>
       <c r="L18" s="86"/>
     </row>
     <row r="19" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
@@ -32682,16 +32682,16 @@
     </row>
     <row r="28" spans="1:22" s="18" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A28" s="21"/>
-      <c r="B28" s="177"/>
-      <c r="C28" s="178"/>
-      <c r="D28" s="178"/>
-      <c r="E28" s="178"/>
-      <c r="F28" s="178"/>
-      <c r="G28" s="178"/>
-      <c r="H28" s="178"/>
-      <c r="I28" s="178"/>
-      <c r="J28" s="178"/>
-      <c r="K28" s="179"/>
+      <c r="B28" s="180"/>
+      <c r="C28" s="181"/>
+      <c r="D28" s="181"/>
+      <c r="E28" s="181"/>
+      <c r="F28" s="181"/>
+      <c r="G28" s="181"/>
+      <c r="H28" s="181"/>
+      <c r="I28" s="181"/>
+      <c r="J28" s="181"/>
+      <c r="K28" s="182"/>
       <c r="L28" s="20"/>
       <c r="M28" s="19"/>
       <c r="N28" s="19"/>
@@ -36660,6 +36660,13 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B28:K28"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:K16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:K18"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="D15:K15"/>
     <mergeCell ref="A3:K3"/>
@@ -36673,13 +36680,6 @@
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="D14:K14"/>
-    <mergeCell ref="B28:K28"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:K16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:K18"/>
   </mergeCells>
   <conditionalFormatting sqref="K64">
     <cfRule type="cellIs" dxfId="5" priority="3" stopIfTrue="1" operator="between">
@@ -36760,32 +36760,32 @@
       <c r="K2" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="54.75" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A3" s="180" t="s">
+      <c r="A3" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="181"/>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
-      <c r="E3" s="181"/>
-      <c r="F3" s="181"/>
-      <c r="G3" s="181"/>
-      <c r="H3" s="181"/>
-      <c r="I3" s="181"/>
-      <c r="J3" s="181"/>
-      <c r="K3" s="181"/>
+      <c r="B3" s="184"/>
+      <c r="C3" s="184"/>
+      <c r="D3" s="184"/>
+      <c r="E3" s="184"/>
+      <c r="F3" s="184"/>
+      <c r="G3" s="184"/>
+      <c r="H3" s="184"/>
+      <c r="I3" s="184"/>
+      <c r="J3" s="184"/>
+      <c r="K3" s="184"/>
     </row>
     <row r="4" spans="1:15" s="46" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="182" t="s">
+      <c r="B4" s="185" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="182"/>
-      <c r="D4" s="182"/>
-      <c r="E4" s="182"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
+      <c r="F4" s="185"/>
+      <c r="G4" s="185"/>
       <c r="H4" s="47" t="s">
         <v>14</v>
       </c>
@@ -36801,12 +36801,12 @@
     </row>
     <row r="5" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A5" s="45"/>
-      <c r="B5" s="183"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
-      <c r="E5" s="184"/>
-      <c r="F5" s="184"/>
-      <c r="G5" s="185"/>
+      <c r="B5" s="186"/>
+      <c r="C5" s="187"/>
+      <c r="D5" s="187"/>
+      <c r="E5" s="187"/>
+      <c r="F5" s="187"/>
+      <c r="G5" s="188"/>
       <c r="H5" s="44"/>
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
@@ -36814,12 +36814,12 @@
     </row>
     <row r="6" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A6" s="45"/>
-      <c r="B6" s="183"/>
-      <c r="C6" s="184"/>
-      <c r="D6" s="184"/>
-      <c r="E6" s="184"/>
-      <c r="F6" s="184"/>
-      <c r="G6" s="185"/>
+      <c r="B6" s="186"/>
+      <c r="C6" s="187"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="187"/>
+      <c r="G6" s="188"/>
       <c r="H6" s="44"/>
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
@@ -36827,12 +36827,12 @@
     </row>
     <row r="7" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A7" s="45"/>
-      <c r="B7" s="183"/>
-      <c r="C7" s="184"/>
-      <c r="D7" s="184"/>
-      <c r="E7" s="184"/>
-      <c r="F7" s="184"/>
-      <c r="G7" s="185"/>
+      <c r="B7" s="186"/>
+      <c r="C7" s="187"/>
+      <c r="D7" s="187"/>
+      <c r="E7" s="187"/>
+      <c r="F7" s="187"/>
+      <c r="G7" s="188"/>
       <c r="H7" s="44"/>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
@@ -36840,12 +36840,12 @@
     </row>
     <row r="8" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A8" s="45"/>
-      <c r="B8" s="183"/>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
-      <c r="F8" s="184"/>
-      <c r="G8" s="185"/>
+      <c r="B8" s="186"/>
+      <c r="C8" s="187"/>
+      <c r="D8" s="187"/>
+      <c r="E8" s="187"/>
+      <c r="F8" s="187"/>
+      <c r="G8" s="188"/>
       <c r="H8" s="44"/>
       <c r="I8" s="43"/>
       <c r="J8" s="43"/>
@@ -36853,12 +36853,12 @@
     </row>
     <row r="9" spans="1:15" s="41" customFormat="1" ht="20.100000000000001" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A9" s="45"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="184"/>
-      <c r="D9" s="184"/>
-      <c r="E9" s="184"/>
-      <c r="F9" s="184"/>
-      <c r="G9" s="185"/>
+      <c r="B9" s="186"/>
+      <c r="C9" s="187"/>
+      <c r="D9" s="187"/>
+      <c r="E9" s="187"/>
+      <c r="F9" s="187"/>
+      <c r="G9" s="188"/>
       <c r="H9" s="44"/>
       <c r="I9" s="43"/>
       <c r="J9" s="43"/>
@@ -36906,117 +36906,117 @@
     </row>
     <row r="13" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A13" s="87"/>
-      <c r="B13" s="186" t="s">
+      <c r="B13" s="179" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="186"/>
-      <c r="D13" s="188" t="str">
+      <c r="C13" s="179"/>
+      <c r="D13" s="178" t="str">
         <f>PyFlange_Gap30deg!D13</f>
         <v>SP2200052</v>
       </c>
-      <c r="E13" s="188"/>
-      <c r="F13" s="188"/>
-      <c r="G13" s="188"/>
-      <c r="H13" s="188"/>
-      <c r="I13" s="188"/>
-      <c r="J13" s="188"/>
-      <c r="K13" s="188"/>
+      <c r="E13" s="178"/>
+      <c r="F13" s="178"/>
+      <c r="G13" s="178"/>
+      <c r="H13" s="178"/>
+      <c r="I13" s="178"/>
+      <c r="J13" s="178"/>
+      <c r="K13" s="178"/>
       <c r="L13" s="86"/>
     </row>
     <row r="14" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A14" s="87"/>
-      <c r="B14" s="186" t="s">
+      <c r="B14" s="179" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="186"/>
-      <c r="D14" s="188" t="str">
+      <c r="C14" s="179"/>
+      <c r="D14" s="178" t="str">
         <f>PyFlange_Gap30deg!D14</f>
         <v>Stichting GROW</v>
       </c>
-      <c r="E14" s="188"/>
-      <c r="F14" s="188"/>
-      <c r="G14" s="188"/>
-      <c r="H14" s="188"/>
-      <c r="I14" s="188"/>
-      <c r="J14" s="188"/>
-      <c r="K14" s="188"/>
+      <c r="E14" s="178"/>
+      <c r="F14" s="178"/>
+      <c r="G14" s="178"/>
+      <c r="H14" s="178"/>
+      <c r="I14" s="178"/>
+      <c r="J14" s="178"/>
+      <c r="K14" s="178"/>
       <c r="L14" s="86"/>
     </row>
     <row r="15" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A15" s="87"/>
-      <c r="B15" s="186" t="s">
+      <c r="B15" s="179" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="186"/>
-      <c r="D15" s="188" t="str">
+      <c r="C15" s="179"/>
+      <c r="D15" s="178" t="str">
         <f>PyFlange_Gap30deg!D15</f>
         <v>Bolt and Beautiful</v>
       </c>
-      <c r="E15" s="188"/>
-      <c r="F15" s="188"/>
-      <c r="G15" s="188"/>
-      <c r="H15" s="188"/>
-      <c r="I15" s="188"/>
-      <c r="J15" s="188"/>
-      <c r="K15" s="188"/>
+      <c r="E15" s="178"/>
+      <c r="F15" s="178"/>
+      <c r="G15" s="178"/>
+      <c r="H15" s="178"/>
+      <c r="I15" s="178"/>
+      <c r="J15" s="178"/>
+      <c r="K15" s="178"/>
       <c r="L15" s="86"/>
     </row>
     <row r="16" spans="1:15" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A16" s="87"/>
-      <c r="B16" s="186" t="s">
+      <c r="B16" s="179" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="186"/>
-      <c r="D16" s="188" t="str">
+      <c r="C16" s="179"/>
+      <c r="D16" s="178" t="str">
         <f>Title</f>
         <v>Flange Segment Analytical Model for 120° gap size</v>
       </c>
-      <c r="E16" s="188"/>
-      <c r="F16" s="188"/>
-      <c r="G16" s="188"/>
-      <c r="H16" s="188"/>
-      <c r="I16" s="188"/>
-      <c r="J16" s="188"/>
-      <c r="K16" s="188"/>
+      <c r="E16" s="178"/>
+      <c r="F16" s="178"/>
+      <c r="G16" s="178"/>
+      <c r="H16" s="178"/>
+      <c r="I16" s="178"/>
+      <c r="J16" s="178"/>
+      <c r="K16" s="178"/>
       <c r="L16" s="86"/>
       <c r="M16" s="88"/>
     </row>
     <row r="17" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A17" s="87"/>
-      <c r="B17" s="186" t="s">
+      <c r="B17" s="179" t="s">
         <v>96</v>
       </c>
-      <c r="C17" s="186"/>
-      <c r="D17" s="188" t="str">
+      <c r="C17" s="179"/>
+      <c r="D17" s="178" t="str">
         <f>PyFlange_Gap30deg!D17</f>
         <v>0.10</v>
       </c>
-      <c r="E17" s="188"/>
-      <c r="F17" s="188"/>
-      <c r="G17" s="188"/>
-      <c r="H17" s="188"/>
-      <c r="I17" s="188"/>
-      <c r="J17" s="188"/>
-      <c r="K17" s="188"/>
+      <c r="E17" s="178"/>
+      <c r="F17" s="178"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="178"/>
+      <c r="I17" s="178"/>
+      <c r="J17" s="178"/>
+      <c r="K17" s="178"/>
       <c r="L17" s="86"/>
     </row>
     <row r="18" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A18" s="87"/>
-      <c r="B18" s="186" t="s">
+      <c r="B18" s="179" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="186"/>
-      <c r="D18" s="187">
+      <c r="C18" s="179"/>
+      <c r="D18" s="189">
         <f>PyFlange_Gap30deg!D18</f>
         <v>45432</v>
       </c>
-      <c r="E18" s="187"/>
-      <c r="F18" s="187"/>
-      <c r="G18" s="187"/>
-      <c r="H18" s="187"/>
-      <c r="I18" s="187"/>
-      <c r="J18" s="187"/>
-      <c r="K18" s="187"/>
+      <c r="E18" s="189"/>
+      <c r="F18" s="189"/>
+      <c r="G18" s="189"/>
+      <c r="H18" s="189"/>
+      <c r="I18" s="189"/>
+      <c r="J18" s="189"/>
+      <c r="K18" s="189"/>
       <c r="L18" s="86"/>
     </row>
     <row r="19" spans="1:22" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
@@ -37204,16 +37204,16 @@
     </row>
     <row r="28" spans="1:22" s="18" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A28" s="21"/>
-      <c r="B28" s="177"/>
-      <c r="C28" s="178"/>
-      <c r="D28" s="178"/>
-      <c r="E28" s="178"/>
-      <c r="F28" s="178"/>
-      <c r="G28" s="178"/>
-      <c r="H28" s="178"/>
-      <c r="I28" s="178"/>
-      <c r="J28" s="178"/>
-      <c r="K28" s="179"/>
+      <c r="B28" s="180"/>
+      <c r="C28" s="181"/>
+      <c r="D28" s="181"/>
+      <c r="E28" s="181"/>
+      <c r="F28" s="181"/>
+      <c r="G28" s="181"/>
+      <c r="H28" s="181"/>
+      <c r="I28" s="181"/>
+      <c r="J28" s="181"/>
+      <c r="K28" s="182"/>
       <c r="L28" s="20"/>
       <c r="M28" s="19"/>
       <c r="N28" s="19"/>
@@ -41182,6 +41182,13 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B28:K28"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:K16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:K17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:K18"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="D15:K15"/>
     <mergeCell ref="A3:K3"/>
@@ -41195,13 +41202,6 @@
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="D14:K14"/>
-    <mergeCell ref="B28:K28"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:K16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:K17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:K18"/>
   </mergeCells>
   <conditionalFormatting sqref="K64">
     <cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="between">
@@ -58996,6 +58996,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="2278e7f3-5df8-4100-b836-5320443b7544" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004E5A98ECA1EC044BB77E0D7F6ADEF7BC" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5e88349ac6f5efd4674595e2a92e1fa9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2278e7f3-5df8-4100-b836-5320443b7544" xmlns:ns4="3fb9cbd1-4a98-4945-a235-2d8a3d5ec2be" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bde21b231255bb48ab8a6ec7dd561648" ns3:_="" ns4:_="">
     <xsd:import namespace="2278e7f3-5df8-4100-b836-5320443b7544"/>
@@ -59248,38 +59265,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="2278e7f3-5df8-4100-b836-5320443b7544" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7863D2-B6F1-4C67-B9E9-1F3A9276C4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52E10DE4-EB42-4EC5-8AEE-EE77FE7979AC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2278e7f3-5df8-4100-b836-5320443b7544"/>
-    <ds:schemaRef ds:uri="3fb9cbd1-4a98-4945-a235-2d8a3d5ec2be"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -59302,9 +59291,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52E10DE4-EB42-4EC5-8AEE-EE77FE7979AC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A7863D2-B6F1-4C67-B9E9-1F3A9276C4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2278e7f3-5df8-4100-b836-5320443b7544"/>
+    <ds:schemaRef ds:uri="3fb9cbd1-4a98-4945-a235-2d8a3d5ec2be"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>